<commit_message>
import des ticket et ses items
</commit_message>
<xml_diff>
--- a/To do/todo.xlsx
+++ b/To do/todo.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
-  <workbookPr/>
+  <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\S6\Modele To DO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eccc9ba13b5ec9e0/Documents/GitHub/Evaluation-glpi-NewApp/To do/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E8D96FC-AE55-4FCB-B1AA-7D5ECEB5EBE0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="groupe" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="21" r:id="rId6"/>
+    <pivotCache cacheId="39" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="71">
   <si>
     <t>Ligne</t>
   </si>
@@ -79,54 +79,15 @@
     <t>Backoffice</t>
   </si>
   <si>
-    <t>Gestion Login</t>
-  </si>
-  <si>
-    <t>Index</t>
-  </si>
-  <si>
-    <t>Création html</t>
-  </si>
-  <si>
     <t>Affichage</t>
   </si>
   <si>
-    <t>Design css</t>
-  </si>
-  <si>
     <t>Metier</t>
   </si>
   <si>
-    <t>checkLogin</t>
-  </si>
-  <si>
     <t>Integration</t>
   </si>
   <si>
-    <t>Gestion Categorie</t>
-  </si>
-  <si>
-    <t>Categorie</t>
-  </si>
-  <si>
-    <t>table login</t>
-  </si>
-  <si>
-    <t>données test</t>
-  </si>
-  <si>
-    <t>Liste</t>
-  </si>
-  <si>
-    <t>Categorie-add</t>
-  </si>
-  <si>
-    <t>Ajout</t>
-  </si>
-  <si>
-    <t>Base</t>
-  </si>
-  <si>
     <t>Total général</t>
   </si>
   <si>
@@ -173,6 +134,126 @@
   </si>
   <si>
     <t>Gestion Reset</t>
+  </si>
+  <si>
+    <t>deleteView</t>
+  </si>
+  <si>
+    <t>Bouton de reinitialisaton</t>
+  </si>
+  <si>
+    <t>deleteService</t>
+  </si>
+  <si>
+    <t>deleteAll</t>
+  </si>
+  <si>
+    <t>Gestion Import</t>
+  </si>
+  <si>
+    <t>importView</t>
+  </si>
+  <si>
+    <t>Formulaire de fichier csv</t>
+  </si>
+  <si>
+    <t>importService</t>
+  </si>
+  <si>
+    <t>importAssets</t>
+  </si>
+  <si>
+    <t>importImage</t>
+  </si>
+  <si>
+    <t>Gestion Protection</t>
+  </si>
+  <si>
+    <t>entreView</t>
+  </si>
+  <si>
+    <t>formulaire de code unique</t>
+  </si>
+  <si>
+    <t>entreService</t>
+  </si>
+  <si>
+    <t>validerCode</t>
+  </si>
+  <si>
+    <t>Gestion Dashboard</t>
+  </si>
+  <si>
+    <t>nombre general d element et ticket</t>
+  </si>
+  <si>
+    <t>dashboardService</t>
+  </si>
+  <si>
+    <t>dashboardView</t>
+  </si>
+  <si>
+    <t>countElement</t>
+  </si>
+  <si>
+    <t>countTicket</t>
+  </si>
+  <si>
+    <t>Gestion Ticket</t>
+  </si>
+  <si>
+    <t>ticketListView</t>
+  </si>
+  <si>
+    <t>liste des tickets</t>
+  </si>
+  <si>
+    <t>ticketService</t>
+  </si>
+  <si>
+    <t>getAllTicket</t>
+  </si>
+  <si>
+    <t>fiche d un ticket</t>
+  </si>
+  <si>
+    <t>ticketFicheView</t>
+  </si>
+  <si>
+    <t>getById</t>
+  </si>
+  <si>
+    <t>Frontoffice</t>
+  </si>
+  <si>
+    <t>Gestion Assets</t>
+  </si>
+  <si>
+    <t>assetsListView</t>
+  </si>
+  <si>
+    <t>liste des elements</t>
+  </si>
+  <si>
+    <t>assetsService</t>
+  </si>
+  <si>
+    <t>getItems</t>
+  </si>
+  <si>
+    <t>recherche multi critere</t>
+  </si>
+  <si>
+    <t>searchAssets</t>
+  </si>
+  <si>
+    <t>ticketformView</t>
+  </si>
+  <si>
+    <t>formulaire de creation de ticket</t>
+  </si>
+  <si>
+    <t>insertTicket</t>
   </si>
 </sst>
 </file>
@@ -182,7 +263,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -223,12 +304,6 @@
       <name val="Liberation Serif"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color theme="1"/>
@@ -262,6 +337,19 @@
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -289,7 +377,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -429,11 +517,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
@@ -453,29 +552,27 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="10" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="10" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" pivotButton="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
@@ -494,6 +591,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -516,7 +619,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Ericka Harimalala" refreshedDate="46178.531826273145" refreshedVersion="7" recordCount="32" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Ericka Harimalala" refreshedDate="46178.741894444443" refreshedVersion="7" recordCount="32" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="B1:K993" sheet="liste des taches"/>
   </cacheSource>
@@ -550,13 +653,13 @@
       <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="5" maxValue="50"/>
     </cacheField>
     <cacheField name="Temps passé" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="90"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="75"/>
     </cacheField>
     <cacheField name="Reste à faire" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="40"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="-25" maxValue="50"/>
     </cacheField>
     <cacheField name="Avancement" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1"/>
+      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1.8"/>
     </cacheField>
   </cacheFields>
   <extLst>
@@ -572,374 +675,374 @@
   <r>
     <s v="Backoffice"/>
     <s v="Gestion Reset"/>
-    <m/>
-    <s v="Création html"/>
+    <s v="deleteView"/>
+    <s v="Bouton de reinitialisaton"/>
     <s v="Affichage"/>
     <x v="0"/>
-    <n v="30"/>
-    <n v="20"/>
-    <n v="10"/>
-    <n v="0.66666666666666663"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Login"/>
-    <s v="Index"/>
-    <s v="Design css"/>
-    <s v="Metier"/>
-    <x v="0"/>
-    <n v="20"/>
-    <n v="0"/>
-    <n v="20"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Login"/>
-    <s v="Index"/>
-    <s v="checkLogin"/>
-    <s v="Integration"/>
-    <x v="0"/>
-    <n v="30"/>
-    <n v="10"/>
-    <n v="20"/>
-    <n v="0.33333333333333331"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie"/>
-    <s v="table login"/>
-    <s v="Affichage"/>
-    <x v="0"/>
-    <n v="10"/>
-    <n v="0"/>
-    <n v="10"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie"/>
-    <s v="données test"/>
-    <s v="Metier"/>
-    <x v="0"/>
-    <n v="50"/>
-    <n v="10"/>
-    <n v="40"/>
-    <n v="0.2"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie"/>
-    <s v="Liste"/>
-    <s v="Integration"/>
-    <x v="0"/>
-    <n v="25"/>
-    <n v="0"/>
-    <n v="25"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
-    <s v="Affichage"/>
-    <x v="0"/>
-    <n v="10"/>
-    <n v="90"/>
+    <n v="5"/>
+    <n v="5"/>
     <n v="0"/>
     <n v="1"/>
   </r>
   <r>
     <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
+    <s v="Gestion Reset"/>
+    <s v="deleteService"/>
+    <s v="deleteAll"/>
     <s v="Metier"/>
     <x v="0"/>
-    <n v="5"/>
-    <n v="30"/>
+    <n v="20"/>
+    <n v="20"/>
     <n v="0"/>
     <n v="1"/>
   </r>
   <r>
     <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
-    <s v="Base"/>
+    <s v="Gestion Reset"/>
+    <s v="deleteView"/>
+    <s v="Bouton de reinitialisaton"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importView"/>
+    <s v="Formulaire de fichier csv"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="15"/>
+    <n v="0"/>
+    <n v="1"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importService"/>
+    <s v="importAssets"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="50"/>
+    <n v="75"/>
+    <n v="-25"/>
+    <n v="1.5"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importService"/>
+    <s v="importAssets"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importService"/>
+    <s v="importAssets"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importService"/>
+    <s v="importImage"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+    <n v="50"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Import"/>
+    <s v="importView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="0"/>
+    <n v="15"/>
+    <n v="0"/>
+  </r>
+  <r>
+    <s v="Backoffice"/>
+    <s v="Gestion Protection"/>
+    <s v="entreView"/>
+    <s v="formulaire de code unique"/>
+    <s v="Affichage"/>
     <x v="0"/>
     <n v="5"/>
-    <n v="0"/>
     <n v="5"/>
     <n v="0"/>
+    <n v="1"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Protection"/>
+    <s v="entreService"/>
+    <s v="validerCode"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="20"/>
+    <n v="20"/>
+    <n v="0"/>
+    <n v="1"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Protection"/>
+    <s v="entreView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="9"/>
+    <n v="-4"/>
+    <n v="1.8"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Dashboard"/>
+    <s v="dashboardView"/>
+    <s v="nombre general d element et ticket"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Dashboard"/>
+    <s v="dashboardService"/>
+    <s v="countElement"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Dashboard"/>
+    <s v="dashboardService"/>
+    <s v="countTicket"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Dashboard"/>
+    <s v="dashboardView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketListView"/>
+    <s v="liste des tickets"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketService"/>
+    <s v="getAllTicket"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketListView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="0"/>
+    <n v="5"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketFicheView"/>
+    <s v="fiche d un ticket"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketService"/>
+    <s v="getById"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Backoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketFicheView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="0"/>
+    <n v="5"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsListView"/>
+    <s v="liste des elements"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="0"/>
+    <n v="15"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsService"/>
+    <s v="getItems"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="20"/>
+    <n v="0"/>
+    <n v="20"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsListView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="10"/>
+    <n v="0"/>
+    <n v="10"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsListView"/>
+    <s v="recherche multi critere"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="0"/>
+    <n v="5"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsService"/>
+    <s v="searchAssets"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="25"/>
+    <n v="0"/>
+    <n v="25"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Assets"/>
+    <s v="assetsListView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="5"/>
+    <n v="0"/>
+    <n v="5"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketformView"/>
+    <s v="formulaire de creation de ticket"/>
+    <s v="Affichage"/>
+    <x v="0"/>
+    <n v="20"/>
+    <n v="0"/>
+    <n v="20"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketService"/>
+    <s v="insertTicket"/>
+    <s v="Metier"/>
+    <x v="0"/>
+    <n v="20"/>
+    <n v="0"/>
+    <n v="20"/>
+    <n v="0"/>
   </r>
   <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="1"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
+    <s v="Frontoffice"/>
+    <s v="Gestion Ticket"/>
+    <s v="ticketformView"/>
+    <s v="Integration"/>
+    <s v="Integration"/>
+    <x v="0"/>
+    <n v="15"/>
+    <n v="0"/>
+    <n v="15"/>
+    <n v="0"/>
   </r>
   <r>
     <m/>
@@ -957,7 +1060,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Recap" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="7" compact="0" compactData="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Recap" cacheId="39" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="7" compact="0" compactData="0">
   <location ref="A1:D5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField name="Catégorie" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
@@ -1229,10 +1332,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1308,33 +1411,35 @@
       <c r="B2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="43" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="6"/>
+      <c r="C2" s="41" t="s">
+        <v>30</v>
+      </c>
+      <c r="D2" s="41" t="s">
+        <v>31</v>
+      </c>
       <c r="E2" s="7" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" s="43" t="s">
-        <v>41</v>
+        <v>12</v>
+      </c>
+      <c r="G2" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H2" s="6">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="I2" s="9">
         <f>detail_avancement!B2</f>
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="J2" s="9">
-        <f t="shared" ref="J2:J7" si="0">H2-I2</f>
-        <v>10</v>
+        <f t="shared" ref="J2:J32" si="0">H2-I2</f>
+        <v>0</v>
       </c>
       <c r="K2" s="10">
-        <f t="shared" ref="K2:K10" si="1">(I2/(I2+J2))</f>
-        <v>0.66666666666666663</v>
+        <f t="shared" ref="K2:K32" si="1">(I2/(I2+J2))</f>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="12.75">
@@ -1345,34 +1450,34 @@
         <v>11</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="43" t="s">
-        <v>41</v>
+      <c r="G3" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H3" s="6">
         <v>20</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="11">
         <f>detail_avancement!B3</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="9">
-        <f t="shared" si="0"/>
         <v>20</v>
+      </c>
+      <c r="J3" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="K3" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="12.75">
@@ -1383,34 +1488,34 @@
         <v>11</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>13</v>
+        <v>30</v>
+      </c>
+      <c r="D4" s="42" t="s">
+        <v>31</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G4" s="43" t="s">
-        <v>41</v>
+        <v>14</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H4" s="6">
-        <v>30</v>
-      </c>
-      <c r="I4" s="9">
+        <v>10</v>
+      </c>
+      <c r="I4" s="11">
         <f>detail_avancement!B4</f>
         <v>10</v>
       </c>
-      <c r="J4" s="9">
-        <f t="shared" si="0"/>
-        <v>20</v>
+      <c r="J4" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="K4" s="10">
         <f t="shared" si="1"/>
-        <v>0.33333333333333331</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="12.75">
@@ -1421,34 +1526,34 @@
         <v>11</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>36</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="6">
         <v>15</v>
       </c>
-      <c r="G5" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="6">
-        <v>10</v>
-      </c>
-      <c r="I5" s="9">
+      <c r="I5" s="11">
         <f>detail_avancement!B5</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="9">
-        <f t="shared" si="0"/>
-        <v>10</v>
+        <v>15</v>
+      </c>
+      <c r="J5" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
       <c r="K5" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="12.75">
@@ -1459,34 +1564,34 @@
         <v>11</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>38</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="43" t="s">
-        <v>41</v>
+        <v>13</v>
+      </c>
+      <c r="G6" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H6" s="6">
         <v>50</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="11">
         <f>detail_avancement!B6</f>
-        <v>10</v>
-      </c>
-      <c r="J6" s="9">
-        <f t="shared" si="0"/>
-        <v>40</v>
+        <v>75</v>
+      </c>
+      <c r="J6" s="11">
+        <f t="shared" si="0"/>
+        <v>-25</v>
       </c>
       <c r="K6" s="10">
         <f t="shared" si="1"/>
-        <v>0.2</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="12.75">
@@ -1497,30 +1602,30 @@
         <v>11</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>21</v>
+        <v>35</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>38</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="43" t="s">
-        <v>41</v>
+        <v>13</v>
+      </c>
+      <c r="G7" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H7" s="6">
-        <v>25</v>
-      </c>
-      <c r="I7" s="9">
+        <v>50</v>
+      </c>
+      <c r="I7" s="11">
         <f>detail_avancement!B7</f>
         <v>0</v>
       </c>
-      <c r="J7" s="9">
-        <f t="shared" si="0"/>
-        <v>25</v>
+      <c r="J7" s="11">
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="K7" s="10">
         <f t="shared" si="1"/>
@@ -1535,33 +1640,34 @@
         <v>11</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>38</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="43" t="s">
-        <v>41</v>
+        <v>13</v>
+      </c>
+      <c r="G8" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H8" s="6">
-        <v>10</v>
-      </c>
-      <c r="I8" s="9">
+        <v>50</v>
+      </c>
+      <c r="I8" s="11">
         <f>detail_avancement!B8</f>
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="J8" s="11">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="K8" s="10">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="12.75">
@@ -1572,33 +1678,34 @@
         <v>11</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>38</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G9" s="43" t="s">
-        <v>41</v>
+        <v>13</v>
+      </c>
+      <c r="G9" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H9" s="6">
-        <v>5</v>
-      </c>
-      <c r="I9" s="9">
+        <v>50</v>
+      </c>
+      <c r="I9" s="11">
         <f>detail_avancement!B9</f>
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="J9" s="11">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>50</v>
       </c>
       <c r="K9" s="10">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="12.75">
@@ -1609,245 +1716,871 @@
         <v>11</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>25</v>
+        <v>35</v>
+      </c>
+      <c r="D10" s="42" t="s">
+        <v>36</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="43" t="s">
-        <v>41</v>
+        <v>14</v>
+      </c>
+      <c r="F10" s="42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" s="41" t="s">
+        <v>28</v>
       </c>
       <c r="H10" s="6">
-        <v>5</v>
-      </c>
-      <c r="I10" s="9">
+        <v>15</v>
+      </c>
+      <c r="I10" s="11">
         <f>detail_avancement!B10</f>
         <v>0</v>
       </c>
-      <c r="J10" s="9">
-        <f>H10-I10</f>
-        <v>5</v>
+      <c r="J10" s="11">
+        <f t="shared" si="0"/>
+        <v>15</v>
       </c>
       <c r="K10" s="10">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" ht="12.75">
       <c r="A11" s="5">
         <v>10</v>
       </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="12"/>
-      <c r="K11" s="12"/>
-    </row>
-    <row r="12" spans="1:11">
+      <c r="B11" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" s="12">
+        <v>5</v>
+      </c>
+      <c r="I11" s="11">
+        <f>detail_avancement!B11</f>
+        <v>5</v>
+      </c>
+      <c r="J11" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="12.75">
       <c r="A12" s="5">
         <v>11</v>
       </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="12"/>
-      <c r="K12" s="12"/>
+      <c r="B12" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="12">
+        <v>20</v>
+      </c>
+      <c r="I12" s="11">
+        <f>detail_avancement!B12</f>
+        <v>20</v>
+      </c>
+      <c r="J12" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K12" s="10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:11" ht="12.75">
       <c r="A13" s="5">
         <v>12</v>
       </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="12"/>
-      <c r="K13" s="12"/>
+      <c r="B13" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" s="44" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H13" s="12">
+        <v>5</v>
+      </c>
+      <c r="I13" s="11">
+        <f>detail_avancement!B13</f>
+        <v>9</v>
+      </c>
+      <c r="J13" s="11">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="K13" s="10">
+        <f t="shared" si="1"/>
+        <v>1.8</v>
+      </c>
     </row>
     <row r="14" spans="1:11" ht="12.75">
       <c r="A14" s="5">
         <v>13</v>
       </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="12"/>
-      <c r="K14" s="12"/>
+      <c r="B14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>47</v>
+      </c>
+      <c r="F14" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H14" s="12">
+        <v>10</v>
+      </c>
+      <c r="I14" s="11">
+        <f>detail_avancement!B14</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K14" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:11" ht="12.75">
       <c r="A15" s="5">
         <v>14</v>
       </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="12"/>
-      <c r="K15" s="12"/>
+      <c r="B15" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="12">
+        <v>10</v>
+      </c>
+      <c r="I15" s="11">
+        <f>detail_avancement!B15</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K15" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:11" ht="12.75">
       <c r="A16" s="5">
         <v>15</v>
       </c>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="12"/>
-      <c r="K16" s="12"/>
+      <c r="B16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="44" t="s">
+        <v>48</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>51</v>
+      </c>
+      <c r="F16" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H16" s="12">
+        <v>10</v>
+      </c>
+      <c r="I16" s="11">
+        <f>detail_avancement!B16</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K16" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:11" ht="12.75">
       <c r="A17" s="5">
         <v>16</v>
       </c>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="12"/>
-      <c r="K17" s="12"/>
+      <c r="B17" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="44" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="12">
+        <v>10</v>
+      </c>
+      <c r="I17" s="11">
+        <f>detail_avancement!B17</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K17" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" spans="1:11" ht="12.75">
       <c r="A18" s="5">
         <v>17</v>
       </c>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="12"/>
-      <c r="K18" s="12"/>
+      <c r="B18" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="F18" s="44" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H18" s="12">
+        <v>10</v>
+      </c>
+      <c r="I18" s="11">
+        <f>detail_avancement!B18</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K18" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:11" ht="12.75">
       <c r="A19" s="5">
         <v>18</v>
       </c>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="12"/>
-      <c r="K19" s="12"/>
+      <c r="B19" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="44" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="12">
+        <v>10</v>
+      </c>
+      <c r="I19" s="11">
+        <f>detail_avancement!B19</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K19" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" spans="1:11" ht="12.75">
       <c r="A20" s="5">
         <v>19</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="12"/>
-      <c r="K20" s="12"/>
+      <c r="B20" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="12">
+        <v>5</v>
+      </c>
+      <c r="I20" s="11">
+        <f>detail_avancement!B20</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K20" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1">
       <c r="A21" s="5">
         <v>20</v>
       </c>
+      <c r="B21" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D21" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="F21" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H21" s="45">
+        <v>10</v>
+      </c>
+      <c r="I21" s="11">
+        <f>detail_avancement!B21</f>
+        <v>0</v>
+      </c>
+      <c r="J21" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K21" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1">
       <c r="A22" s="5">
         <v>21</v>
       </c>
+      <c r="B22" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="F22" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H22" s="45">
+        <v>10</v>
+      </c>
+      <c r="I22" s="11">
+        <f>detail_avancement!B22</f>
+        <v>0</v>
+      </c>
+      <c r="J22" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K22" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1">
       <c r="A23" s="5">
         <v>22</v>
       </c>
+      <c r="B23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="44" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="45" t="s">
+        <v>58</v>
+      </c>
+      <c r="E23" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H23" s="45">
+        <v>5</v>
+      </c>
+      <c r="I23" s="11">
+        <f>detail_avancement!B23</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K23" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1">
       <c r="A24" s="5">
         <v>23</v>
       </c>
+      <c r="B24" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C24" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="D24" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="E24" s="45" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H24" s="45">
+        <v>15</v>
+      </c>
+      <c r="I24" s="11">
+        <f>detail_avancement!B24</f>
+        <v>0</v>
+      </c>
+      <c r="J24" s="11">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="K24" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1">
       <c r="A25" s="5">
         <v>24</v>
       </c>
+      <c r="B25" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="45" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="45" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H25" s="45">
+        <v>20</v>
+      </c>
+      <c r="I25" s="11">
+        <f>detail_avancement!B25</f>
+        <v>0</v>
+      </c>
+      <c r="J25" s="11">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="K25" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1">
       <c r="A26" s="5">
         <v>25</v>
       </c>
+      <c r="B26" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C26" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="E26" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H26" s="45">
+        <v>10</v>
+      </c>
+      <c r="I26" s="11">
+        <f>detail_avancement!B26</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="11">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="K26" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1">
       <c r="A27" s="5">
         <v>26</v>
       </c>
+      <c r="B27" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="45" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G27" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H27" s="47">
+        <v>5</v>
+      </c>
+      <c r="I27" s="11">
+        <f>detail_avancement!B27</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K27" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" spans="1:11" ht="15.75" customHeight="1">
       <c r="A28" s="5">
         <v>27</v>
       </c>
+      <c r="B28" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="45" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" s="45" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="45" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H28" s="47">
+        <v>25</v>
+      </c>
+      <c r="I28" s="11">
+        <f>detail_avancement!B28</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="11">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="K28" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" spans="1:11" ht="15.75" customHeight="1">
       <c r="A29" s="5">
         <v>28</v>
+      </c>
+      <c r="B29" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="47" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="45" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H29" s="47">
+        <v>5</v>
+      </c>
+      <c r="I29" s="11">
+        <f>detail_avancement!B29</f>
+        <v>0</v>
+      </c>
+      <c r="J29" s="11">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="K29" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="15.75" customHeight="1">
       <c r="A30" s="5">
         <v>29</v>
       </c>
+      <c r="B30" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" s="45" t="s">
+        <v>69</v>
+      </c>
+      <c r="F30" s="47" t="s">
+        <v>12</v>
+      </c>
+      <c r="G30" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H30" s="47">
+        <v>20</v>
+      </c>
+      <c r="I30" s="11">
+        <f>detail_avancement!B30</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="11">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="K30" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" spans="1:11" ht="15.75" customHeight="1">
       <c r="A31" s="5">
         <v>30</v>
       </c>
+      <c r="B31" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="D31" s="45" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="45" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H31" s="47">
+        <v>20</v>
+      </c>
+      <c r="I31" s="11">
+        <f>detail_avancement!B31</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="11">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="K31" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" spans="1:11" ht="15.75" customHeight="1">
       <c r="A32" s="5">
         <v>31</v>
       </c>
+      <c r="B32" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="47" t="s">
+        <v>52</v>
+      </c>
+      <c r="D32" s="45" t="s">
+        <v>68</v>
+      </c>
+      <c r="E32" s="45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" s="47" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" s="41" t="s">
+        <v>28</v>
+      </c>
+      <c r="H32" s="47">
+        <v>15</v>
+      </c>
+      <c r="I32" s="11">
+        <f>detail_avancement!B32</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="11">
+        <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="K32" s="10">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:1" ht="15.75" customHeight="1">
       <c r="A33" s="5">
@@ -2080,8 +2813,9 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="13" type="noConversion"/>
+  <phoneticPr fontId="12" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2094,62 +2828,65 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="26"/>
-      <c r="B1" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="28"/>
-      <c r="D1" s="29"/>
+      <c r="A1" s="24"/>
+      <c r="B1" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="26"/>
+      <c r="D1" s="27"/>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2" s="31" t="s">
-        <v>39</v>
+      <c r="B2" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="29" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="32">
-        <v>185</v>
-      </c>
-      <c r="C3" s="33">
-        <v>160</v>
-      </c>
-      <c r="D3" s="34">
-        <v>130</v>
+      <c r="A3" s="24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="30">
+        <v>520</v>
+      </c>
+      <c r="C3" s="31">
+        <v>159</v>
+      </c>
+      <c r="D3" s="32">
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="35" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" s="36"/>
-      <c r="C4" s="37"/>
-      <c r="D4" s="38"/>
+      <c r="A4" s="33" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="34"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="36"/>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="39" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="40">
-        <v>185</v>
-      </c>
-      <c r="C5" s="41">
-        <v>160</v>
-      </c>
-      <c r="D5" s="42">
-        <v>130</v>
-      </c>
+      <c r="A5" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="38">
+        <v>520</v>
+      </c>
+      <c r="C5" s="39">
+        <v>159</v>
+      </c>
+      <c r="D5" s="40">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" customHeight="1">
+      <c r="B7" s="43"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="13" t="s">
@@ -2157,7 +2894,7 @@
       </c>
       <c r="B12" s="14">
         <f>avancement!D2</f>
-        <v>0.55172413793103448</v>
+        <v>0.30576923076923079</v>
       </c>
     </row>
   </sheetData>
@@ -2182,52 +2919,55 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" customHeight="1">
       <c r="A1" s="15" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15">
       <c r="A2" s="16">
         <f>SUM('liste des taches'!H:H)</f>
-        <v>185</v>
+        <v>520</v>
       </c>
       <c r="B2" s="16">
         <f>SUM('liste des taches'!I:I)</f>
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C2" s="16">
         <f>SUM('liste des taches'!J:J)</f>
-        <v>130</v>
+        <v>361</v>
       </c>
       <c r="D2" s="17">
         <f>(B2/(B2+C2))</f>
-        <v>0.55172413793103448</v>
+        <v>0.30576923076923079</v>
       </c>
       <c r="E2" s="18">
         <f>((B2+C2)-A2)/A2</f>
-        <v>0.56756756756756754</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="19"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="15">
+      <c r="A3" s="19">
+        <f>A2/60</f>
+        <v>8.6666666666666661</v>
+      </c>
       <c r="B3" s="19"/>
       <c r="C3" s="16">
         <f>C2/60</f>
-        <v>2.1666666666666665</v>
+        <v>6.0166666666666666</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E3" s="19"/>
     </row>
@@ -2249,45 +2989,47 @@
         <v>0</v>
       </c>
       <c r="B1" s="21" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="C1" s="22">
-        <v>46048</v>
+        <v>46147</v>
       </c>
       <c r="D1" s="22">
-        <v>46049</v>
+        <v>46148</v>
       </c>
       <c r="E1" s="22">
-        <v>46050</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15">
       <c r="A2" s="23">
         <v>1</v>
       </c>
       <c r="B2" s="16">
-        <f t="shared" ref="B2:B10" si="0">SUM(D2:P2)</f>
-        <v>20</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="23">
-        <v>20</v>
-      </c>
+        <f>SUM(C2:C2)</f>
+        <v>5</v>
+      </c>
+      <c r="C2" s="19">
+        <v>5</v>
+      </c>
+      <c r="D2" s="23"/>
       <c r="E2" s="19"/>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="15">
       <c r="A3" s="23">
         <v>2</v>
       </c>
       <c r="B3" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+        <f t="shared" ref="B3:B26" si="0">SUM(C3:C3)</f>
+        <v>20</v>
+      </c>
+      <c r="C3" s="19">
+        <v>20</v>
+      </c>
+      <c r="D3" s="23"/>
       <c r="E3" s="19"/>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="15">
       <c r="A4" s="23">
         <v>3</v>
       </c>
@@ -2296,40 +3038,40 @@
         <v>10</v>
       </c>
       <c r="C4" s="23">
-        <v>20</v>
-      </c>
-      <c r="D4" s="23">
         <v>10</v>
       </c>
+      <c r="D4" s="23"/>
       <c r="E4" s="19"/>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="15">
       <c r="A5" s="23">
         <v>4</v>
       </c>
       <c r="B5" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
+        <v>15</v>
+      </c>
+      <c r="C5" s="19">
+        <v>15</v>
+      </c>
+      <c r="D5" s="23"/>
       <c r="E5" s="19"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="15">
       <c r="A6" s="23">
         <v>5</v>
       </c>
       <c r="B6" s="16">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="24">
-        <v>10</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C6" s="19">
+        <v>75</v>
+      </c>
+      <c r="D6" s="23"/>
       <c r="E6" s="19"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" ht="15">
       <c r="A7" s="23">
         <v>6</v>
       </c>
@@ -2338,21 +3080,19 @@
         <v>0</v>
       </c>
       <c r="C7" s="19"/>
-      <c r="D7" s="19"/>
+      <c r="D7" s="23"/>
       <c r="E7" s="19"/>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" ht="15">
       <c r="A8" s="23">
         <v>7</v>
       </c>
       <c r="B8" s="16">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="C8" s="19"/>
-      <c r="D8" s="24">
-        <v>90</v>
-      </c>
+      <c r="D8" s="23"/>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="15">
@@ -2361,11 +3101,9 @@
       </c>
       <c r="B9" s="16">
         <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="D9" s="25">
-        <v>30</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D9" s="23"/>
     </row>
     <row r="10" spans="1:5" ht="15">
       <c r="A10" s="23">
@@ -2380,80 +3118,153 @@
       <c r="A11" s="23">
         <v>10</v>
       </c>
+      <c r="B11" s="16">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" customHeight="1">
       <c r="A12" s="23">
         <v>11</v>
       </c>
+      <c r="B12" s="16">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="C12">
+        <v>20</v>
+      </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" customHeight="1">
       <c r="A13" s="23">
         <v>12</v>
       </c>
+      <c r="B13" s="16">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="C13">
+        <v>9</v>
+      </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" customHeight="1">
       <c r="A14" s="23">
         <v>13</v>
       </c>
+      <c r="B14" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1">
       <c r="A15" s="23">
         <v>14</v>
       </c>
+      <c r="B15" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1">
       <c r="A16" s="23">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B16" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" customHeight="1">
       <c r="A17" s="23">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B17" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" customHeight="1">
       <c r="A18" s="23">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B18" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15.75" customHeight="1">
       <c r="A19" s="23">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B19" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15.75" customHeight="1">
       <c r="A20" s="23">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B20" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15.75" customHeight="1">
       <c r="A21" s="23">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B21" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15.75" customHeight="1">
       <c r="A22" s="23">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B22" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15.75" customHeight="1">
       <c r="A23" s="23">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B23" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15.75" customHeight="1">
       <c r="A24" s="23">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B24" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15.75" customHeight="1">
       <c r="A25" s="23">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" ht="15.75" customHeight="1">
+      <c r="B25" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15.75" customHeight="1">
       <c r="A26" s="23">
         <v>25</v>
+      </c>
+      <c r="B26" s="16">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
import tout ou rien
</commit_message>
<xml_diff>
--- a/To do/todo.xlsx
+++ b/To do/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eccc9ba13b5ec9e0/Documents/GitHub/Evaluation-glpi-NewApp/To do/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E8D96FC-AE55-4FCB-B1AA-7D5ECEB5EBE0}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD7A1935-FF93-4CB3-BC0D-F183651B4323}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="groupe" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="39" r:id="rId6"/>
+    <pivotCache cacheId="3" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="73">
   <si>
     <t>Ligne</t>
   </si>
@@ -254,6 +254,12 @@
   </si>
   <si>
     <t>insertTicket</t>
+  </si>
+  <si>
+    <t>importTicktes</t>
+  </si>
+  <si>
+    <t>importCost</t>
   </si>
 </sst>
 </file>
@@ -619,7 +625,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Ericka Harimalala" refreshedDate="46178.741894444443" refreshedVersion="7" recordCount="32" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Ericka Harimalala" refreshedDate="46178.907231597223" refreshedVersion="7" recordCount="32" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="B1:K993" sheet="liste des taches"/>
   </cacheSource>
@@ -643,10 +649,10 @@
       <sharedItems containsBlank="1" count="6">
         <s v="ETU003350"/>
         <m/>
+        <s v="ETU00WWWW" u="1"/>
+        <s v="ETU00ZZZZ" u="1"/>
+        <s v="ETU00YYYY" u="1"/>
         <s v="ETU00XXXX" u="1"/>
-        <s v="ETU00ZZZZ" u="1"/>
-        <s v="ETU00WWWW" u="1"/>
-        <s v="ETU00YYYY" u="1"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Estimation" numFmtId="0">
@@ -1060,7 +1066,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Recap" cacheId="39" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="7" compact="0" compactData="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Recap" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="7" compact="0" compactData="0">
   <location ref="A1:D5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="10">
     <pivotField name="Catégorie" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
@@ -1071,9 +1077,9 @@
     <pivotField name="Qui" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
       <items count="7">
         <item x="0"/>
-        <item m="1" x="4"/>
         <item m="1" x="2"/>
         <item m="1" x="5"/>
+        <item m="1" x="4"/>
         <item m="1" x="3"/>
         <item x="1"/>
         <item t="default"/>
@@ -1360,7 +1366,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:K78"/>
+  <dimension ref="A1:L78"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
@@ -1369,7 +1375,7 @@
     <col min="5" max="5" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1">
+    <row r="1" spans="1:12" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1404,7 +1410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="12.75">
+    <row r="2" spans="1:12" ht="12.75">
       <c r="A2" s="5">
         <v>1</v>
       </c>
@@ -1441,8 +1447,12 @@
         <f t="shared" ref="K2:K32" si="1">(I2/(I2+J2))</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="12.75">
+      <c r="L2">
+        <f>SUM(J:J)</f>
+        <v>146</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="12.75">
       <c r="A3" s="5">
         <v>2</v>
       </c>
@@ -1480,7 +1490,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="12.75">
+    <row r="4" spans="1:12" ht="12.75">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -1518,7 +1528,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="12.75">
+    <row r="5" spans="1:12" ht="12.75">
       <c r="A5" s="5">
         <v>4</v>
       </c>
@@ -1556,7 +1566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="12.75">
+    <row r="6" spans="1:12" ht="12.75">
       <c r="A6" s="5">
         <v>5</v>
       </c>
@@ -1594,7 +1604,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="12.75">
+    <row r="7" spans="1:12" ht="12.75">
       <c r="A7" s="5">
         <v>6</v>
       </c>
@@ -1608,7 +1618,7 @@
         <v>38</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="F7" s="8" t="s">
         <v>13</v>
@@ -1621,18 +1631,18 @@
       </c>
       <c r="I7" s="11">
         <f>detail_avancement!B7</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="J7" s="11">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>-25</v>
       </c>
       <c r="K7" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="12.75">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="12.75">
       <c r="A8" s="5">
         <v>7</v>
       </c>
@@ -1646,7 +1656,7 @@
         <v>38</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>39</v>
+        <v>72</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>13</v>
@@ -1659,18 +1669,18 @@
       </c>
       <c r="I8" s="11">
         <f>detail_avancement!B8</f>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="J8" s="11">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>-25</v>
       </c>
       <c r="K8" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="12.75">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="12.75">
       <c r="A9" s="5">
         <v>8</v>
       </c>
@@ -1697,18 +1707,18 @@
       </c>
       <c r="I9" s="11">
         <f>detail_avancement!B9</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J9" s="11">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="K9" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="12.75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="12.75">
       <c r="A10" s="5">
         <v>9</v>
       </c>
@@ -1735,18 +1745,18 @@
       </c>
       <c r="I10" s="11">
         <f>detail_avancement!B10</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J10" s="11">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K10" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="12.75">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="12.75">
       <c r="A11" s="5">
         <v>10</v>
       </c>
@@ -1784,7 +1794,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="12.75">
+    <row r="12" spans="1:12" ht="12.75">
       <c r="A12" s="5">
         <v>11</v>
       </c>
@@ -1822,7 +1832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="12.75">
+    <row r="13" spans="1:12" ht="12.75">
       <c r="A13" s="5">
         <v>12</v>
       </c>
@@ -1860,7 +1870,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="12.75">
+    <row r="14" spans="1:12" ht="12.75">
       <c r="A14" s="5">
         <v>13</v>
       </c>
@@ -1898,7 +1908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="12.75">
+    <row r="15" spans="1:12" ht="12.75">
       <c r="A15" s="5">
         <v>14</v>
       </c>
@@ -1936,7 +1946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="12.75">
+    <row r="16" spans="1:12" ht="12.75">
       <c r="A16" s="5">
         <v>15</v>
       </c>
@@ -2827,7 +2837,7 @@
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" ht="12.75">
       <c r="A1" s="24"/>
       <c r="B1" s="25" t="s">
         <v>23</v>
@@ -2835,7 +2845,7 @@
       <c r="C1" s="26"/>
       <c r="D1" s="27"/>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" ht="12.75">
       <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
@@ -2849,7 +2859,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" ht="12.75">
       <c r="A3" s="24" t="s">
         <v>28</v>
       </c>
@@ -2863,7 +2873,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" ht="12.75">
       <c r="A4" s="33" t="s">
         <v>27</v>
       </c>
@@ -2871,7 +2881,7 @@
       <c r="C4" s="35"/>
       <c r="D4" s="36"/>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" ht="12.75">
       <c r="A5" s="37" t="s">
         <v>15</v>
       </c>
@@ -2888,13 +2898,13 @@
     <row r="7" spans="1:4" ht="15.75" customHeight="1">
       <c r="B7" s="43"/>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" ht="12.75">
       <c r="A12" s="13" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="14">
         <f>avancement!D2</f>
-        <v>0.30576923076923079</v>
+        <v>0.71923076923076923</v>
       </c>
     </row>
   </sheetData>
@@ -2941,15 +2951,15 @@
       </c>
       <c r="B2" s="16">
         <f>SUM('liste des taches'!I:I)</f>
-        <v>159</v>
+        <v>374</v>
       </c>
       <c r="C2" s="16">
         <f>SUM('liste des taches'!J:J)</f>
-        <v>361</v>
+        <v>146</v>
       </c>
       <c r="D2" s="17">
         <f>(B2/(B2+C2))</f>
-        <v>0.30576923076923079</v>
+        <v>0.71923076923076923</v>
       </c>
       <c r="E2" s="18">
         <f>((B2+C2)-A2)/A2</f>
@@ -2964,7 +2974,7 @@
       <c r="B3" s="19"/>
       <c r="C3" s="16">
         <f>C2/60</f>
-        <v>6.0166666666666666</v>
+        <v>2.4333333333333331</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>21</v>
@@ -3006,7 +3016,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="16">
-        <f>SUM(C2:C2)</f>
+        <f>SUM(C2:K2)</f>
         <v>5</v>
       </c>
       <c r="C2" s="19">
@@ -3020,7 +3030,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="16">
-        <f t="shared" ref="B3:B26" si="0">SUM(C3:C3)</f>
+        <f t="shared" ref="B3:B26" si="0">SUM(C3:K3)</f>
         <v>20</v>
       </c>
       <c r="C3" s="19">
@@ -3077,10 +3087,12 @@
       </c>
       <c r="B7" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C7" s="19"/>
-      <c r="D7" s="23"/>
+      <c r="D7" s="23">
+        <v>75</v>
+      </c>
       <c r="E7" s="19"/>
     </row>
     <row r="8" spans="1:5" ht="15">
@@ -3089,10 +3101,12 @@
       </c>
       <c r="B8" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="C8" s="19"/>
-      <c r="D8" s="23"/>
+      <c r="D8" s="23">
+        <v>75</v>
+      </c>
       <c r="E8" s="19"/>
     </row>
     <row r="9" spans="1:5" ht="15">
@@ -3101,9 +3115,12 @@
       </c>
       <c r="B9" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D9" s="23"/>
+      <c r="E9">
+        <v>50</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="15">
       <c r="A10" s="23">
@@ -3111,7 +3128,11 @@
       </c>
       <c r="B10" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>15</v>
+      </c>
+      <c r="D10" s="23"/>
+      <c r="E10">
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
liste des tickets et fiche ticket
</commit_message>
<xml_diff>
--- a/To do/todo.xlsx
+++ b/To do/todo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/eccc9ba13b5ec9e0/Documents/GitHub/Evaluation-glpi-NewApp/To do/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD7A1935-FF93-4CB3-BC0D-F183651B4323}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{54828E04-CEAF-42A4-922D-53BC2D354A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{797F826C-50C0-48FD-9F99-457371F74632}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="groupe" sheetId="1" r:id="rId1"/>
@@ -1449,7 +1449,7 @@
       </c>
       <c r="L2">
         <f>SUM(J:J)</f>
-        <v>146</v>
+        <v>-19</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="12.75">
@@ -1897,15 +1897,15 @@
       </c>
       <c r="I14" s="11">
         <f>detail_avancement!B14</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J14" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K14" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="12.75">
@@ -1935,15 +1935,15 @@
       </c>
       <c r="I15" s="11">
         <f>detail_avancement!B15</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J15" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>-40</v>
       </c>
       <c r="K15" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="12.75">
@@ -1973,15 +1973,15 @@
       </c>
       <c r="I16" s="11">
         <f>detail_avancement!B16</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J16" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>-10</v>
       </c>
       <c r="K16" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="12.75">
@@ -2011,15 +2011,15 @@
       </c>
       <c r="I17" s="11">
         <f>detail_avancement!B17</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J17" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K17" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="12.75">
@@ -2049,15 +2049,15 @@
       </c>
       <c r="I18" s="11">
         <f>detail_avancement!B18</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J18" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K18" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="12.75">
@@ -2087,15 +2087,15 @@
       </c>
       <c r="I19" s="11">
         <f>detail_avancement!B19</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J19" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K19" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="12.75">
@@ -2125,15 +2125,15 @@
       </c>
       <c r="I20" s="11">
         <f>detail_avancement!B20</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J20" s="11">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K20" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1">
@@ -2163,15 +2163,15 @@
       </c>
       <c r="I21" s="11">
         <f>detail_avancement!B21</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="J21" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>-10</v>
       </c>
       <c r="K21" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1">
@@ -2201,15 +2201,15 @@
       </c>
       <c r="I22" s="11">
         <f>detail_avancement!B22</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="J22" s="11">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K22" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1">
@@ -2239,15 +2239,15 @@
       </c>
       <c r="I23" s="11">
         <f>detail_avancement!B23</f>
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="J23" s="11">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>-20</v>
       </c>
       <c r="K23" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1">
@@ -2904,7 +2904,7 @@
       </c>
       <c r="B12" s="14">
         <f>avancement!D2</f>
-        <v>0.71923076923076923</v>
+        <v>1.0365384615384616</v>
       </c>
     </row>
   </sheetData>
@@ -2951,15 +2951,15 @@
       </c>
       <c r="B2" s="16">
         <f>SUM('liste des taches'!I:I)</f>
-        <v>374</v>
+        <v>539</v>
       </c>
       <c r="C2" s="16">
         <f>SUM('liste des taches'!J:J)</f>
-        <v>146</v>
+        <v>-19</v>
       </c>
       <c r="D2" s="17">
         <f>(B2/(B2+C2))</f>
-        <v>0.71923076923076923</v>
+        <v>1.0365384615384616</v>
       </c>
       <c r="E2" s="18">
         <f>((B2+C2)-A2)/A2</f>
@@ -2974,7 +2974,7 @@
       <c r="B3" s="19"/>
       <c r="C3" s="16">
         <f>C2/60</f>
-        <v>2.4333333333333331</v>
+        <v>-0.31666666666666665</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>21</v>
@@ -3177,7 +3177,10 @@
       </c>
       <c r="B14" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" customHeight="1">
@@ -3186,7 +3189,10 @@
       </c>
       <c r="B15" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>50</v>
+      </c>
+      <c r="E15">
+        <v>50</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1">
@@ -3195,73 +3201,97 @@
       </c>
       <c r="B16" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15.75" customHeight="1">
+        <v>20</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" customHeight="1">
       <c r="A17" s="23">
         <v>16</v>
       </c>
       <c r="B17" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="15.75" customHeight="1">
       <c r="A18" s="23">
         <v>17</v>
       </c>
       <c r="B18" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15.75" customHeight="1">
+        <v>10</v>
+      </c>
+      <c r="E18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" customHeight="1">
       <c r="A19" s="23">
         <v>18</v>
       </c>
       <c r="B19" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15.75" customHeight="1">
+        <v>10</v>
+      </c>
+      <c r="E19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" customHeight="1">
       <c r="A20" s="23">
         <v>19</v>
       </c>
       <c r="B20" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15.75" customHeight="1">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="15.75" customHeight="1">
       <c r="A21" s="23">
         <v>20</v>
       </c>
       <c r="B21" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15.75" customHeight="1">
+        <v>20</v>
+      </c>
+      <c r="E21">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1">
       <c r="A22" s="23">
         <v>21</v>
       </c>
       <c r="B22" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15.75" customHeight="1">
+        <v>10</v>
+      </c>
+      <c r="E22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="15.75" customHeight="1">
       <c r="A23" s="23">
         <v>22</v>
       </c>
       <c r="B23" s="16">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15.75" customHeight="1">
+        <v>25</v>
+      </c>
+      <c r="E23">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="15.75" customHeight="1">
       <c r="A24" s="23">
         <v>23</v>
       </c>
@@ -3270,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="15.75" customHeight="1">
+    <row r="25" spans="1:5" ht="15.75" customHeight="1">
       <c r="A25" s="23">
         <v>24</v>
       </c>
@@ -3279,7 +3309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="15.75" customHeight="1">
+    <row r="26" spans="1:5" ht="15.75" customHeight="1">
       <c r="A26" s="23">
         <v>25</v>
       </c>

</xml_diff>